<commit_message>
Add Phase 1 MVP Administrative AI Agent; compress roadmap to 5 months
</commit_message>
<xml_diff>
--- a/AI_Agent_Programme_Plan.xlsx
+++ b/AI_Agent_Programme_Plan.xlsx
@@ -724,24 +724,17 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Enterprise AI Agent Programme - Delivery Roadmap (AWS, 12 Months)</t>
+          <t>Enterprise AI Agent Programme - Delivery Roadmap (AWS, 5 Months)</t>
         </is>
       </c>
     </row>
@@ -793,41 +786,6 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>M7</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>M8</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>M9</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -842,25 +800,18 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>M1-M2</t>
-        </is>
-      </c>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n"/>
       <c r="F5" s="8" t="n"/>
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="n"/>
-      <c r="N5" s="8" t="n"/>
-      <c r="O5" s="8" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -870,30 +821,23 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="n"/>
       <c r="G6" s="8" t="n"/>
       <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
-      <c r="M6" s="8" t="n"/>
-      <c r="N6" s="8" t="n"/>
-      <c r="O6" s="8" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -903,30 +847,23 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>M4-M5</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
-      <c r="N7" s="8" t="n"/>
-      <c r="O7" s="8" t="n"/>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>M2-M3</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -936,30 +873,23 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>M3-M4</t>
+        </is>
+      </c>
       <c r="H8" s="8" t="n"/>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>M6-M7</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="n"/>
-      <c r="M8" s="8" t="n"/>
-      <c r="N8" s="8" t="n"/>
-      <c r="O8" s="8" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -969,30 +899,23 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
       <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
       <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>M8-M9</t>
-        </is>
-      </c>
-      <c r="L9" s="12" t="inlineStr"/>
-      <c r="M9" s="8" t="n"/>
-      <c r="N9" s="8" t="n"/>
-      <c r="O9" s="8" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1002,30 +925,23 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>M12</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
       <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
-      <c r="L10" s="8" t="n"/>
-      <c r="M10" s="13" t="inlineStr"/>
-      <c r="N10" s="13" t="inlineStr">
-        <is>
-          <t>M10-M12</t>
-        </is>
-      </c>
-      <c r="O10" s="13" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>M4-M5</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr"/>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -1035,30 +951,23 @@
       </c>
       <c r="B12" s="15" t="n"/>
       <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>MVP live</t>
         </is>
       </c>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Gov insights</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Knowledge Q&amp;A</t>
+        </is>
+      </c>
       <c r="H12" s="16" t="inlineStr">
-        <is>
-          <t>Gov insights</t>
-        </is>
-      </c>
-      <c r="I12" s="15" t="n"/>
-      <c r="J12" s="15" t="n"/>
-      <c r="K12" s="15" t="n"/>
-      <c r="L12" s="16" t="inlineStr">
-        <is>
-          <t>Knowledge Q&amp;A</t>
-        </is>
-      </c>
-      <c r="M12" s="15" t="n"/>
-      <c r="N12" s="15" t="n"/>
-      <c r="O12" s="16" t="inlineStr">
         <is>
           <t>Control Tower</t>
         </is>
@@ -1143,12 +1052,12 @@
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>M1 - M2</t>
+          <t>M1 - M1</t>
         </is>
       </c>
       <c r="C2" s="20" t="inlineStr">
         <is>
-          <t>2 mo</t>
+          <t>1 mo</t>
         </is>
       </c>
       <c r="D2" s="20" t="inlineStr">
@@ -1187,7 +1096,7 @@
       </c>
       <c r="B3" s="22" t="inlineStr">
         <is>
-          <t>M3 - M3</t>
+          <t>M2 - M2</t>
         </is>
       </c>
       <c r="C3" s="22" t="inlineStr">
@@ -1229,7 +1138,7 @@
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>M4 - M5</t>
+          <t>M2 - M3</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
@@ -1271,7 +1180,7 @@
       </c>
       <c r="B5" s="22" t="inlineStr">
         <is>
-          <t>M6 - M7</t>
+          <t>M3 - M4</t>
         </is>
       </c>
       <c r="C5" s="22" t="inlineStr">
@@ -1314,12 +1223,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>M8 - M9</t>
+          <t>M4 - M4</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>2 mo</t>
+          <t>1 mo</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -1355,12 +1264,12 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>M10 - M12</t>
+          <t>M4 - M5</t>
         </is>
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
-          <t>3 mo</t>
+          <t>2 mo</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
@@ -1400,7 +1309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1499,49 +1408,49 @@
       </c>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>M1-M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="C4" s="29" t="inlineStr">
         <is>
-          <t>Prompt + extract action items, owners, due dates (structured JSON)</t>
+          <t>Extract actions/owners/due dates; minutes, summaries, register</t>
         </is>
       </c>
       <c r="D4" s="29" t="inlineStr">
         <is>
-          <t>Amazon Bedrock, Lambda</t>
+          <t>Amazon Bedrock, DynamoDB</t>
         </is>
       </c>
       <c r="E4" s="29" t="inlineStr">
         <is>
-          <t>Structured action data</t>
+          <t>MVP live (minutes + register)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>Generate meeting minutes &amp; summaries; persist action register</t>
-        </is>
-      </c>
-      <c r="D5" s="29" t="inlineStr">
-        <is>
-          <t>Amazon Bedrock, DynamoDB</t>
-        </is>
-      </c>
-      <c r="E5" s="29" t="inlineStr">
-        <is>
-          <t>Minutes, summaries, register</t>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled scan of open/overdue actions; reminder + escalation logic</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>EventBridge, Lambda</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>Automated reminders</t>
         </is>
       </c>
     </row>
@@ -1553,49 +1462,49 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C6" s="31" t="inlineStr">
         <is>
-          <t>Scheduled scan of open/overdue actions; reminder + escalation logic</t>
+          <t>Notification channels and closure-evidence capture</t>
         </is>
       </c>
       <c r="D6" s="31" t="inlineStr">
         <is>
-          <t>EventBridge, Lambda</t>
+          <t>Amazon SES / SNS, S3</t>
         </is>
       </c>
       <c r="E6" s="31" t="inlineStr">
         <is>
-          <t>Automated reminders</t>
+          <t>Alerts &amp; status reports</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="B7" s="31" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="C7" s="31" t="inlineStr">
-        <is>
-          <t>Notification channels and closure-evidence capture</t>
-        </is>
-      </c>
-      <c r="D7" s="31" t="inlineStr">
-        <is>
-          <t>Amazon SES / SNS, S3</t>
-        </is>
-      </c>
-      <c r="E7" s="31" t="inlineStr">
-        <is>
-          <t>Alerts &amp; status reports</t>
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>M2-M3</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Ingest SteerCo/CIO/Cyber/Risk/Audit outputs into knowledge base</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>Bedrock Knowledge Bases, S3</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>Governance corpus</t>
         </is>
       </c>
     </row>
@@ -1607,49 +1516,49 @@
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>Ingest SteerCo/CIO/Cyber/Risk/Audit outputs into knowledge base</t>
+          <t>Theme, risk &amp; dependency detection; executive summaries</t>
         </is>
       </c>
       <c r="D8" s="29" t="inlineStr">
         <is>
-          <t>Bedrock Knowledge Bases, S3</t>
+          <t>Amazon Bedrock, Lambda</t>
         </is>
       </c>
       <c r="E8" s="29" t="inlineStr">
         <is>
-          <t>Governance corpus</t>
+          <t>Risk insights &amp; exec reports</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="32" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>M4-M5</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>Theme, risk &amp; dependency detection; executive summaries</t>
-        </is>
-      </c>
-      <c r="D9" s="29" t="inlineStr">
-        <is>
-          <t>Amazon Bedrock, Lambda</t>
-        </is>
-      </c>
-      <c r="E9" s="29" t="inlineStr">
-        <is>
-          <t>Risk insights &amp; exec reports</t>
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>Build data lake / ETL for reporting; define KPIs &amp; metrics</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>AWS Glue, Athena, S3</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="inlineStr">
+        <is>
+          <t>Curated reporting datasets</t>
         </is>
       </c>
     </row>
@@ -1661,49 +1570,49 @@
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M3-M4</t>
         </is>
       </c>
       <c r="C10" s="31" t="inlineStr">
         <is>
-          <t>Build data lake / ETL for reporting; define KPIs &amp; metrics</t>
+          <t>Dashboards, monthly reports, CIO packs, trend analysis</t>
         </is>
       </c>
       <c r="D10" s="31" t="inlineStr">
         <is>
-          <t>AWS Glue, Athena, S3</t>
+          <t>Amazon QuickSight</t>
         </is>
       </c>
       <c r="E10" s="31" t="inlineStr">
         <is>
-          <t>Curated reporting datasets</t>
+          <t>Executive reporting packs</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="inlineStr">
-        <is>
-          <t>M6-M7</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>Dashboards, monthly reports, CIO packs, trend analysis</t>
-        </is>
-      </c>
-      <c r="D11" s="31" t="inlineStr">
-        <is>
-          <t>Amazon QuickSight</t>
-        </is>
-      </c>
-      <c r="E11" s="31" t="inlineStr">
-        <is>
-          <t>Executive reporting packs</t>
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Index all outputs; build vector store for semantic search</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>OpenSearch Serverless, S3</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>Searchable index</t>
         </is>
       </c>
     </row>
@@ -1715,49 +1624,49 @@
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>Index all outputs; build vector store for semantic search</t>
+          <t>RAG-based Q&amp;A assistant over organisational memory</t>
         </is>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>OpenSearch Serverless, S3</t>
+          <t>Bedrock Knowledge Bases (RAG)</t>
         </is>
       </c>
       <c r="E12" s="29" t="inlineStr">
         <is>
-          <t>Searchable index</t>
+          <t>Natural-language Q&amp;A</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="34" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>M8-M9</t>
-        </is>
-      </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>RAG-based Q&amp;A assistant over organisational memory</t>
-        </is>
-      </c>
-      <c r="D13" s="29" t="inlineStr">
-        <is>
-          <t>Bedrock Knowledge Bases (RAG)</t>
-        </is>
-      </c>
-      <c r="E13" s="29" t="inlineStr">
-        <is>
-          <t>Natural-language Q&amp;A</t>
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>Design orchestration spine; agent registry &amp; shared data contracts</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>Step Functions, API Gateway</t>
+        </is>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Orchestration design</t>
         </is>
       </c>
     </row>
@@ -1769,22 +1678,22 @@
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>Design orchestration spine; agent registry &amp; shared data contracts</t>
+          <t>Wire all agents together; central console &amp; access control</t>
         </is>
       </c>
       <c r="D14" s="31" t="inlineStr">
         <is>
-          <t>Step Functions, API Gateway</t>
+          <t>Bedrock Agents, Cognito</t>
         </is>
       </c>
       <c r="E14" s="31" t="inlineStr">
         <is>
-          <t>Orchestration design</t>
+          <t>Unified platform</t>
         </is>
       </c>
     </row>
@@ -1796,47 +1705,20 @@
       </c>
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>M10-M11</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>Wire all agents together; central console &amp; access control</t>
+          <t>End-to-end testing, hardening, go-live &amp; handover</t>
         </is>
       </c>
       <c r="D15" s="31" t="inlineStr">
         <is>
-          <t>Bedrock Agents, Cognito</t>
+          <t>CloudWatch, Step Functions</t>
         </is>
       </c>
       <c r="E15" s="31" t="inlineStr">
-        <is>
-          <t>Unified platform</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="35" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="B16" s="31" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>End-to-end testing, hardening, go-live &amp; handover</t>
-        </is>
-      </c>
-      <c r="D16" s="31" t="inlineStr">
-        <is>
-          <t>CloudWatch, Step Functions</t>
-        </is>
-      </c>
-      <c r="E16" s="31" t="inlineStr">
         <is>
           <t>Production Control Tower</t>
         </is>

</xml_diff>

<commit_message>
Excel: use actual calendar dates (kickoff 17 Jun 2026, go-live 16 Nov 2026)
</commit_message>
<xml_diff>
--- a/AI_Agent_Programme_Plan.xlsx
+++ b/AI_Agent_Programme_Plan.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,12 +55,6 @@
       <name val="Calibri"/>
       <color rgb="001B2430"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -267,90 +261,90 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -718,30 +712,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Enterprise AI Agent Programme - Delivery Roadmap (AWS, 5 Months)</t>
+          <t>Enterprise AI Agent Programme - Delivery Roadmap (AWS)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>6 Phases - MVP to Central Control Tower</t>
+          <t>Kickoff 17 Jun 2026  -  Go-live 16 Nov 2026  (5-month delivery window)</t>
         </is>
       </c>
     </row>
@@ -763,27 +758,32 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>Jun 2026</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>Jul 2026</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Aug 2026</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>Sep 2026</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
         </is>
       </c>
     </row>
@@ -795,23 +795,20 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>17 Jun</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n"/>
+          <t>16 Jul</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
       <c r="F5" s="8" t="n"/>
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -821,23 +818,20 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>17 Jul</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>16 Aug</t>
         </is>
       </c>
       <c r="D6" s="8" t="n"/>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
       <c r="G6" s="8" t="n"/>
       <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -847,23 +841,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>17 Jul</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>16 Sep</t>
         </is>
       </c>
       <c r="D7" s="8" t="n"/>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>M2-M3</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="8" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
       <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -873,23 +864,20 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>17 Aug</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>16 Oct</t>
         </is>
       </c>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
-      <c r="F8" s="11" t="inlineStr"/>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>M3-M4</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
+      <c r="I8" s="8" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -899,23 +887,20 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>17 Sep</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>16 Oct</t>
         </is>
       </c>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
       <c r="F9" s="8" t="n"/>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="8" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -925,25 +910,22 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>17 Sep</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>16 Nov</t>
         </is>
       </c>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
       <c r="F10" s="8" t="n"/>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>M4-M5</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr"/>
-    </row>
-    <row r="12" ht="26" customHeight="1">
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="13" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Key Milestones</t>
@@ -951,39 +933,44 @@
       </c>
       <c r="B12" s="15" t="n"/>
       <c r="C12" s="15" t="n"/>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>MVP live</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="16" t="inlineStr">
-        <is>
-          <t>Gov insights</t>
-        </is>
-      </c>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>MVP live
+(16 Jul)</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="n"/>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>Knowledge Q&amp;A</t>
+          <t>Governance insights
+(16 Sep)</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>Control Tower</t>
+          <t>Knowledge Q&amp;A
+(16 Oct)</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>Control Tower go-live
+(16 Nov)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>Cross-cutting from M1: Security &amp; IAM, Cost governance, Data privacy/PII, CI/CD, Human-in-the-loop review.</t>
+          <t>Columns are calendar months. Shaded = phase active that month. Cross-cutting from kickoff: Security &amp; IAM, cost governance, data privacy/PII, CI/CD, human-in-the-loop review.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -995,16 +982,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1015,36 +1003,41 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Timeline</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="C1" s="18" t="inlineStr">
         <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="E1" s="18" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="F1" s="18" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="F1" s="18" t="inlineStr">
+      <c r="G1" s="18" t="inlineStr">
         <is>
           <t>Core AWS Services</t>
         </is>
       </c>
-      <c r="G1" s="18" t="inlineStr">
+      <c r="H1" s="18" t="inlineStr">
         <is>
           <t>Key Deliverables</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="70" customHeight="1">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Phase 1 - Administrative AI Agent (MVP)</t>
@@ -1052,25 +1045,30 @@
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>M1 - M1</t>
+          <t>17 Jun 2026</t>
         </is>
       </c>
       <c r="C2" s="20" t="inlineStr">
         <is>
+          <t>16 Jul 2026</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
           <t>1 mo</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="E2" s="20" t="inlineStr">
         <is>
           <t>AI/ML Lead</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="F2" s="20" t="inlineStr">
         <is>
           <t>Automate meeting admin: transcripts to minutes, actions, owners, due dates</t>
         </is>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="G2" s="20" t="inlineStr">
         <is>
           <t>Amazon Transcribe
 Amazon Bedrock
@@ -1079,7 +1077,7 @@
 AWS Lambda</t>
         </is>
       </c>
-      <c r="G2" s="20" t="inlineStr">
+      <c r="H2" s="20" t="inlineStr">
         <is>
           <t>Meeting minutes
 Action register
@@ -1088,7 +1086,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="70" customHeight="1">
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Phase 2 - Action Tracking Agent</t>
@@ -1096,25 +1094,30 @@
       </c>
       <c r="B3" s="22" t="inlineStr">
         <is>
-          <t>M2 - M2</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="C3" s="22" t="inlineStr">
         <is>
+          <t>16 Aug 2026</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="inlineStr">
+        <is>
           <t>1 mo</t>
         </is>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>Automation Eng</t>
         </is>
       </c>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>Monitor, remind, escalate and report on open / overdue actions</t>
         </is>
       </c>
-      <c r="F3" s="22" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Amazon EventBridge
 Amazon SES / SNS
@@ -1122,7 +1125,7 @@
 AWS Lambda</t>
         </is>
       </c>
-      <c r="G3" s="22" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Weekly action reports
 Overdue alerts
@@ -1130,7 +1133,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="70" customHeight="1">
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Phase 3 - Governance &amp; Forum Agent</t>
@@ -1138,25 +1141,30 @@
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>M2 - M3</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
+          <t>16 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
           <t>2 mo</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Data Eng</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>Read SteerCo / CIO / Cyber / Risk / Audit outputs; detect themes &amp; risks</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="G4" s="20" t="inlineStr">
         <is>
           <t>Amazon Bedrock
 Bedrock Knowledge Bases
@@ -1164,7 +1172,7 @@
 AWS Lambda</t>
         </is>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="H4" s="20" t="inlineStr">
         <is>
           <t>Governance dashboard
 Executive reports
@@ -1172,7 +1180,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Phase 4 - Reporting &amp; Analytics Agent</t>
@@ -1180,25 +1188,30 @@
       </c>
       <c r="B5" s="22" t="inlineStr">
         <is>
-          <t>M3 - M4</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="C5" s="22" t="inlineStr">
         <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
           <t>2 mo</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>BI Lead</t>
         </is>
       </c>
-      <c r="E5" s="22" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>Consolidate reports, measure delivery, build CIO packs &amp; trend analysis</t>
         </is>
       </c>
-      <c r="F5" s="22" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Amazon QuickSight
 AWS Glue
@@ -1206,7 +1219,7 @@
 Amazon S3</t>
         </is>
       </c>
-      <c r="G5" s="22" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>QuickSight dashboards
 Monthly reports
@@ -1215,7 +1228,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="70" customHeight="1">
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Phase 5 - Enterprise Knowledge Agent</t>
@@ -1223,32 +1236,37 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>M4 - M4</t>
+          <t>17 Sep 2026</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
           <t>1 mo</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>AI/ML Lead</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="F6" s="20" t="inlineStr">
         <is>
           <t>Searchable organisational memory; natural-language Q&amp;A over all outputs</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="G6" s="20" t="inlineStr">
         <is>
           <t>Bedrock Knowledge Bases
 OpenSearch Serverless
 Amazon Bedrock (RAG)</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="H6" s="20" t="inlineStr">
         <is>
           <t>Searchable knowledge base
 Q&amp;A assistant
@@ -1256,7 +1274,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="70" customHeight="1">
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Phase 6 - Central Control Tower (Orchestration)</t>
@@ -1264,25 +1282,30 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>M4 - M5</t>
+          <t>17 Sep 2026</t>
         </is>
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
+          <t>16 Nov 2026</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
           <t>2 mo</t>
         </is>
       </c>
-      <c r="D7" s="22" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>Solutions Architect</t>
         </is>
       </c>
-      <c r="E7" s="22" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
         <is>
           <t>Connect all agents through a central platform - the "spine"</t>
         </is>
       </c>
-      <c r="F7" s="22" t="inlineStr">
+      <c r="G7" s="22" t="inlineStr">
         <is>
           <t>Amazon Bedrock Agents
 AWS Step Functions
@@ -1290,7 +1313,7 @@
 Amazon Cognito</t>
         </is>
       </c>
-      <c r="G7" s="22" t="inlineStr">
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>Unified orchestration platform
 Agent registry
@@ -1309,14 +1332,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1327,20 +1351,25 @@
       </c>
       <c r="B1" s="27" t="inlineStr">
         <is>
-          <t>Month(s)</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="C1" s="27" t="inlineStr">
         <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
           <t>Workstream / Task</t>
         </is>
       </c>
-      <c r="D1" s="27" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
         <is>
           <t>AWS Service</t>
         </is>
       </c>
-      <c r="E1" s="27" t="inlineStr">
+      <c r="F1" s="27" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
@@ -1354,20 +1383,25 @@
       </c>
       <c r="B2" s="29" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>17 Jun</t>
         </is>
       </c>
       <c r="C2" s="29" t="inlineStr">
         <is>
+          <t>16 Jul</t>
+        </is>
+      </c>
+      <c r="D2" s="29" t="inlineStr">
+        <is>
           <t>Set up AWS landing zone, IAM roles, S3 buckets for raw inputs</t>
         </is>
       </c>
-      <c r="D2" s="29" t="inlineStr">
+      <c r="E2" s="29" t="inlineStr">
         <is>
           <t>S3, IAM, Organizations</t>
         </is>
       </c>
-      <c r="E2" s="29" t="inlineStr">
+      <c r="F2" s="29" t="inlineStr">
         <is>
           <t>Secure ingest foundation</t>
         </is>
@@ -1381,20 +1415,25 @@
       </c>
       <c r="B3" s="29" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>17 Jun</t>
         </is>
       </c>
       <c r="C3" s="29" t="inlineStr">
         <is>
+          <t>16 Jul</t>
+        </is>
+      </c>
+      <c r="D3" s="29" t="inlineStr">
+        <is>
           <t>Transcribe recordings to text; ingest Teams transcripts &amp; notes</t>
         </is>
       </c>
-      <c r="D3" s="29" t="inlineStr">
+      <c r="E3" s="29" t="inlineStr">
         <is>
           <t>Amazon Transcribe, S3</t>
         </is>
       </c>
-      <c r="E3" s="29" t="inlineStr">
+      <c r="F3" s="29" t="inlineStr">
         <is>
           <t>Normalised transcript store</t>
         </is>
@@ -1408,20 +1447,25 @@
       </c>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>17 Jun</t>
         </is>
       </c>
       <c r="C4" s="29" t="inlineStr">
         <is>
+          <t>16 Jul</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
           <t>Extract actions/owners/due dates; minutes, summaries, register</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>Amazon Bedrock, DynamoDB</t>
         </is>
       </c>
-      <c r="E4" s="29" t="inlineStr">
+      <c r="F4" s="29" t="inlineStr">
         <is>
           <t>MVP live (minutes + register)</t>
         </is>
@@ -1435,20 +1479,25 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>17 Jul</t>
         </is>
       </c>
       <c r="C5" s="31" t="inlineStr">
         <is>
+          <t>16 Aug</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
           <t>Scheduled scan of open/overdue actions; reminder + escalation logic</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="E5" s="31" t="inlineStr">
         <is>
           <t>EventBridge, Lambda</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="F5" s="31" t="inlineStr">
         <is>
           <t>Automated reminders</t>
         </is>
@@ -1462,20 +1511,25 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>17 Jul</t>
         </is>
       </c>
       <c r="C6" s="31" t="inlineStr">
         <is>
+          <t>16 Aug</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
           <t>Notification channels and closure-evidence capture</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="E6" s="31" t="inlineStr">
         <is>
           <t>Amazon SES / SNS, S3</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>Alerts &amp; status reports</t>
         </is>
@@ -1489,20 +1543,25 @@
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>M2-M3</t>
+          <t>17 Jul</t>
         </is>
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
+          <t>16 Sep</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
           <t>Ingest SteerCo/CIO/Cyber/Risk/Audit outputs into knowledge base</t>
         </is>
       </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>Bedrock Knowledge Bases, S3</t>
         </is>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="F7" s="29" t="inlineStr">
         <is>
           <t>Governance corpus</t>
         </is>
@@ -1516,20 +1575,25 @@
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>17 Aug</t>
         </is>
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
+          <t>16 Sep</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
           <t>Theme, risk &amp; dependency detection; executive summaries</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>Amazon Bedrock, Lambda</t>
         </is>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="F8" s="29" t="inlineStr">
         <is>
           <t>Risk insights &amp; exec reports</t>
         </is>
@@ -1543,20 +1607,25 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>17 Aug</t>
         </is>
       </c>
       <c r="C9" s="31" t="inlineStr">
         <is>
+          <t>16 Sep</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
           <t>Build data lake / ETL for reporting; define KPIs &amp; metrics</t>
         </is>
       </c>
-      <c r="D9" s="31" t="inlineStr">
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>AWS Glue, Athena, S3</t>
         </is>
       </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>Curated reporting datasets</t>
         </is>
@@ -1570,20 +1639,25 @@
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>M3-M4</t>
+          <t>17 Aug</t>
         </is>
       </c>
       <c r="C10" s="31" t="inlineStr">
         <is>
+          <t>16 Oct</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr">
+        <is>
           <t>Dashboards, monthly reports, CIO packs, trend analysis</t>
         </is>
       </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="E10" s="31" t="inlineStr">
         <is>
           <t>Amazon QuickSight</t>
         </is>
       </c>
-      <c r="E10" s="31" t="inlineStr">
+      <c r="F10" s="31" t="inlineStr">
         <is>
           <t>Executive reporting packs</t>
         </is>
@@ -1597,20 +1671,25 @@
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>17 Sep</t>
         </is>
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
+          <t>16 Oct</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
           <t>Index all outputs; build vector store for semantic search</t>
         </is>
       </c>
-      <c r="D11" s="29" t="inlineStr">
+      <c r="E11" s="29" t="inlineStr">
         <is>
           <t>OpenSearch Serverless, S3</t>
         </is>
       </c>
-      <c r="E11" s="29" t="inlineStr">
+      <c r="F11" s="29" t="inlineStr">
         <is>
           <t>Searchable index</t>
         </is>
@@ -1624,20 +1703,25 @@
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>17 Sep</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
+          <t>16 Oct</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
           <t>RAG-based Q&amp;A assistant over organisational memory</t>
         </is>
       </c>
-      <c r="D12" s="29" t="inlineStr">
+      <c r="E12" s="29" t="inlineStr">
         <is>
           <t>Bedrock Knowledge Bases (RAG)</t>
         </is>
       </c>
-      <c r="E12" s="29" t="inlineStr">
+      <c r="F12" s="29" t="inlineStr">
         <is>
           <t>Natural-language Q&amp;A</t>
         </is>
@@ -1651,20 +1735,25 @@
       </c>
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>17 Sep</t>
         </is>
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
+          <t>16 Oct</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
           <t>Design orchestration spine; agent registry &amp; shared data contracts</t>
         </is>
       </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="E13" s="31" t="inlineStr">
         <is>
           <t>Step Functions, API Gateway</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr">
+      <c r="F13" s="31" t="inlineStr">
         <is>
           <t>Orchestration design</t>
         </is>
@@ -1678,20 +1767,25 @@
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>17 Oct</t>
         </is>
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
+          <t>16 Nov</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
           <t>Wire all agents together; central console &amp; access control</t>
         </is>
       </c>
-      <c r="D14" s="31" t="inlineStr">
+      <c r="E14" s="31" t="inlineStr">
         <is>
           <t>Bedrock Agents, Cognito</t>
         </is>
       </c>
-      <c r="E14" s="31" t="inlineStr">
+      <c r="F14" s="31" t="inlineStr">
         <is>
           <t>Unified platform</t>
         </is>
@@ -1705,20 +1799,25 @@
       </c>
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>17 Oct</t>
         </is>
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
+          <t>16 Nov</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
           <t>End-to-end testing, hardening, go-live &amp; handover</t>
         </is>
       </c>
-      <c r="D15" s="31" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>CloudWatch, Step Functions</t>
         </is>
       </c>
-      <c r="E15" s="31" t="inlineStr">
+      <c r="F15" s="31" t="inlineStr">
         <is>
           <t>Production Control Tower</t>
         </is>

</xml_diff>

<commit_message>
Excel: real date-typed cells + date labels in timeline bars
</commit_message>
<xml_diff>
--- a/AI_Agent_Programme_Plan.xlsx
+++ b/AI_Agent_Programme_Plan.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Tasks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Phase Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Detailed Tasks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,8 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="22">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd mmm yyyy"/>
+  </numFmts>
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +58,12 @@
       <name val="Calibri"/>
       <color rgb="001B2430"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -240,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -257,94 +266,106 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -716,14 +737,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -793,17 +814,17 @@
           <t>Phase 1 - Administrative AI Agent (MVP)</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>17 Jun</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>16 Jul</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n"/>
+      <c r="B5" s="6" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>17 Jun - 16 Jul</t>
+        </is>
+      </c>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="8" t="n"/>
       <c r="G5" s="8" t="n"/>
@@ -816,18 +837,18 @@
           <t>Phase 2 - Action Tracking Agent</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>17 Jul</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>16 Aug</t>
-        </is>
+      <c r="B6" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>46250</v>
       </c>
       <c r="D6" s="8" t="n"/>
-      <c r="E6" s="9" t="n"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>17 Jul - 16 Aug</t>
+        </is>
+      </c>
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="8" t="n"/>
       <c r="H6" s="8" t="n"/>
@@ -839,18 +860,18 @@
           <t>Phase 3 - Governance &amp; Forum Agent</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>17 Jul</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>16 Sep</t>
-        </is>
+      <c r="B7" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>46281</v>
       </c>
       <c r="D7" s="8" t="n"/>
-      <c r="E7" s="10" t="n"/>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>17 Jul - 16 Sep</t>
+        </is>
+      </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="10" t="n"/>
       <c r="H7" s="8" t="n"/>
@@ -862,19 +883,19 @@
           <t>Phase 4 - Reporting &amp; Analytics Agent</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>17 Aug</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
+      <c r="B8" s="6" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>46311</v>
       </c>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
-      <c r="F8" s="11" t="n"/>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>17 Aug - 16 Oct</t>
+        </is>
+      </c>
       <c r="G8" s="11" t="n"/>
       <c r="H8" s="11" t="n"/>
       <c r="I8" s="8" t="n"/>
@@ -885,20 +906,20 @@
           <t>Phase 5 - Enterprise Knowledge Agent</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>17 Sep</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
+      <c r="B9" s="6" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>46311</v>
       </c>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
       <c r="F9" s="8" t="n"/>
-      <c r="G9" s="12" t="n"/>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>17 Sep - 16 Oct</t>
+        </is>
+      </c>
       <c r="H9" s="12" t="n"/>
       <c r="I9" s="8" t="n"/>
     </row>
@@ -908,20 +929,20 @@
           <t>Phase 6 - Central Control Tower (Orchestration)</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>17 Sep</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>16 Nov</t>
-        </is>
+      <c r="B10" s="6" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>46342</v>
       </c>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
       <c r="F10" s="8" t="n"/>
-      <c r="G10" s="13" t="n"/>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>17 Sep - 16 Nov</t>
+        </is>
+      </c>
       <c r="H10" s="13" t="n"/>
       <c r="I10" s="13" t="n"/>
     </row>
@@ -1043,32 +1064,28 @@
           <t>Phase 1 - Administrative AI Agent (MVP)</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
-        <is>
-          <t>17 Jun 2026</t>
-        </is>
-      </c>
-      <c r="C2" s="20" t="inlineStr">
-        <is>
-          <t>16 Jul 2026</t>
-        </is>
-      </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="B2" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C2" s="20" t="n">
+        <v>46219</v>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>1 mo</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>AI/ML Lead</t>
         </is>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
         <is>
           <t>Automate meeting admin: transcripts to minutes, actions, owners, due dates</t>
         </is>
       </c>
-      <c r="G2" s="20" t="inlineStr">
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>Amazon Transcribe
 Amazon Bedrock
@@ -1077,7 +1094,7 @@
 AWS Lambda</t>
         </is>
       </c>
-      <c r="H2" s="20" t="inlineStr">
+      <c r="H2" s="21" t="inlineStr">
         <is>
           <t>Meeting minutes
 Action register
@@ -1087,37 +1104,33 @@
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Phase 2 - Action Tracking Agent</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
-        <is>
-          <t>17 Jul 2026</t>
-        </is>
-      </c>
-      <c r="C3" s="22" t="inlineStr">
-        <is>
-          <t>16 Aug 2026</t>
-        </is>
-      </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="B3" s="23" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C3" s="23" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>1 mo</t>
         </is>
       </c>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Automation Eng</t>
         </is>
       </c>
-      <c r="F3" s="22" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Monitor, remind, escalate and report on open / overdue actions</t>
         </is>
       </c>
-      <c r="G3" s="22" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Amazon EventBridge
 Amazon SES / SNS
@@ -1125,7 +1138,7 @@
 AWS Lambda</t>
         </is>
       </c>
-      <c r="H3" s="22" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>Weekly action reports
 Overdue alerts
@@ -1134,37 +1147,33 @@
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Phase 3 - Governance &amp; Forum Agent</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>17 Jul 2026</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
-        <is>
-          <t>16 Sep 2026</t>
-        </is>
-      </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="B4" s="20" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C4" s="20" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>2 mo</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Data Eng</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>Read SteerCo / CIO / Cyber / Risk / Audit outputs; detect themes &amp; risks</t>
         </is>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>Amazon Bedrock
 Bedrock Knowledge Bases
@@ -1172,7 +1181,7 @@
 AWS Lambda</t>
         </is>
       </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>Governance dashboard
 Executive reports
@@ -1181,37 +1190,33 @@
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Phase 4 - Reporting &amp; Analytics Agent</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>17 Aug 2026</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="inlineStr">
-        <is>
-          <t>16 Oct 2026</t>
-        </is>
-      </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="B5" s="23" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>2 mo</t>
         </is>
       </c>
-      <c r="E5" s="22" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>BI Lead</t>
         </is>
       </c>
-      <c r="F5" s="22" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>Consolidate reports, measure delivery, build CIO packs &amp; trend analysis</t>
         </is>
       </c>
-      <c r="G5" s="22" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Amazon QuickSight
 AWS Glue
@@ -1219,7 +1224,7 @@
 Amazon S3</t>
         </is>
       </c>
-      <c r="H5" s="22" t="inlineStr">
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>QuickSight dashboards
 Monthly reports
@@ -1229,44 +1234,40 @@
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Phase 5 - Enterprise Knowledge Agent</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>17 Sep 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>16 Oct 2026</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="B6" s="20" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>1 mo</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>AI/ML Lead</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>Searchable organisational memory; natural-language Q&amp;A over all outputs</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>Bedrock Knowledge Bases
 OpenSearch Serverless
 Amazon Bedrock (RAG)</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>Searchable knowledge base
 Q&amp;A assistant
@@ -1275,37 +1276,33 @@
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Phase 6 - Central Control Tower (Orchestration)</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
-        <is>
-          <t>17 Sep 2026</t>
-        </is>
-      </c>
-      <c r="C7" s="22" t="inlineStr">
-        <is>
-          <t>16 Nov 2026</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="inlineStr">
+      <c r="B7" s="23" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>46342</v>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>2 mo</t>
         </is>
       </c>
-      <c r="E7" s="22" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Solutions Architect</t>
         </is>
       </c>
-      <c r="F7" s="22" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>Connect all agents through a central platform - the "spine"</t>
         </is>
       </c>
-      <c r="G7" s="22" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Amazon Bedrock Agents
 AWS Step Functions
@@ -1313,7 +1310,7 @@
 Amazon Cognito</t>
         </is>
       </c>
-      <c r="H7" s="22" t="inlineStr">
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>Unified orchestration platform
 Agent registry
@@ -1336,488 +1333,432 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B1" s="27" t="inlineStr">
+      <c r="B1" s="29" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C1" s="27" t="inlineStr">
+      <c r="C1" s="29" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="D1" s="27" t="inlineStr">
+      <c r="D1" s="29" t="inlineStr">
         <is>
           <t>Workstream / Task</t>
         </is>
       </c>
-      <c r="E1" s="27" t="inlineStr">
+      <c r="E1" s="29" t="inlineStr">
         <is>
           <t>AWS Service</t>
         </is>
       </c>
-      <c r="F1" s="27" t="inlineStr">
+      <c r="F1" s="29" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B2" s="29" t="inlineStr">
-        <is>
-          <t>17 Jun</t>
-        </is>
-      </c>
-      <c r="C2" s="29" t="inlineStr">
-        <is>
-          <t>16 Jul</t>
-        </is>
-      </c>
-      <c r="D2" s="29" t="inlineStr">
+      <c r="B2" s="31" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C2" s="31" t="n">
+        <v>46219</v>
+      </c>
+      <c r="D2" s="32" t="inlineStr">
         <is>
           <t>Set up AWS landing zone, IAM roles, S3 buckets for raw inputs</t>
         </is>
       </c>
-      <c r="E2" s="29" t="inlineStr">
+      <c r="E2" s="32" t="inlineStr">
         <is>
           <t>S3, IAM, Organizations</t>
         </is>
       </c>
-      <c r="F2" s="29" t="inlineStr">
+      <c r="F2" s="32" t="inlineStr">
         <is>
           <t>Secure ingest foundation</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B3" s="29" t="inlineStr">
-        <is>
-          <t>17 Jun</t>
-        </is>
-      </c>
-      <c r="C3" s="29" t="inlineStr">
-        <is>
-          <t>16 Jul</t>
-        </is>
-      </c>
-      <c r="D3" s="29" t="inlineStr">
+      <c r="B3" s="31" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C3" s="31" t="n">
+        <v>46219</v>
+      </c>
+      <c r="D3" s="32" t="inlineStr">
         <is>
           <t>Transcribe recordings to text; ingest Teams transcripts &amp; notes</t>
         </is>
       </c>
-      <c r="E3" s="29" t="inlineStr">
+      <c r="E3" s="32" t="inlineStr">
         <is>
           <t>Amazon Transcribe, S3</t>
         </is>
       </c>
-      <c r="F3" s="29" t="inlineStr">
+      <c r="F3" s="32" t="inlineStr">
         <is>
           <t>Normalised transcript store</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
-        <is>
-          <t>17 Jun</t>
-        </is>
-      </c>
-      <c r="C4" s="29" t="inlineStr">
-        <is>
-          <t>16 Jul</t>
-        </is>
-      </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="B4" s="31" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C4" s="31" t="n">
+        <v>46219</v>
+      </c>
+      <c r="D4" s="32" t="inlineStr">
         <is>
           <t>Extract actions/owners/due dates; minutes, summaries, register</t>
         </is>
       </c>
-      <c r="E4" s="29" t="inlineStr">
+      <c r="E4" s="32" t="inlineStr">
         <is>
           <t>Amazon Bedrock, DynamoDB</t>
         </is>
       </c>
-      <c r="F4" s="29" t="inlineStr">
+      <c r="F4" s="32" t="inlineStr">
         <is>
           <t>MVP live (minutes + register)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
-        <is>
-          <t>17 Jul</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>16 Aug</t>
-        </is>
-      </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="B5" s="34" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C5" s="34" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
         <is>
           <t>Scheduled scan of open/overdue actions; reminder + escalation logic</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="35" t="inlineStr">
         <is>
           <t>EventBridge, Lambda</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="F5" s="35" t="inlineStr">
         <is>
           <t>Automated reminders</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
-        <is>
-          <t>17 Jul</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>16 Aug</t>
-        </is>
-      </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="B6" s="34" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C6" s="34" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>Notification channels and closure-evidence capture</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="E6" s="35" t="inlineStr">
         <is>
           <t>Amazon SES / SNS, S3</t>
         </is>
       </c>
-      <c r="F6" s="31" t="inlineStr">
+      <c r="F6" s="35" t="inlineStr">
         <is>
           <t>Alerts &amp; status reports</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>Phase 3</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
-        <is>
-          <t>17 Jul</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>16 Sep</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="B7" s="31" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C7" s="31" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
         <is>
           <t>Ingest SteerCo/CIO/Cyber/Risk/Audit outputs into knowledge base</t>
         </is>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="32" t="inlineStr">
         <is>
           <t>Bedrock Knowledge Bases, S3</t>
         </is>
       </c>
-      <c r="F7" s="29" t="inlineStr">
+      <c r="F7" s="32" t="inlineStr">
         <is>
           <t>Governance corpus</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="36" t="inlineStr">
         <is>
           <t>Phase 3</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>17 Aug</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>16 Sep</t>
-        </is>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="B8" s="31" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C8" s="31" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
         <is>
           <t>Theme, risk &amp; dependency detection; executive summaries</t>
         </is>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="32" t="inlineStr">
         <is>
           <t>Amazon Bedrock, Lambda</t>
         </is>
       </c>
-      <c r="F8" s="29" t="inlineStr">
+      <c r="F8" s="32" t="inlineStr">
         <is>
           <t>Risk insights &amp; exec reports</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>Phase 4</t>
         </is>
       </c>
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>17 Aug</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>16 Sep</t>
-        </is>
-      </c>
-      <c r="D9" s="31" t="inlineStr">
+      <c r="B9" s="34" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C9" s="34" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
         <is>
           <t>Build data lake / ETL for reporting; define KPIs &amp; metrics</t>
         </is>
       </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="E9" s="35" t="inlineStr">
         <is>
           <t>AWS Glue, Athena, S3</t>
         </is>
       </c>
-      <c r="F9" s="31" t="inlineStr">
+      <c r="F9" s="35" t="inlineStr">
         <is>
           <t>Curated reporting datasets</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>Phase 4</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
-        <is>
-          <t>17 Aug</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
-      </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="B10" s="34" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C10" s="34" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
         <is>
           <t>Dashboards, monthly reports, CIO packs, trend analysis</t>
         </is>
       </c>
-      <c r="E10" s="31" t="inlineStr">
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>Amazon QuickSight</t>
         </is>
       </c>
-      <c r="F10" s="31" t="inlineStr">
+      <c r="F10" s="35" t="inlineStr">
         <is>
           <t>Executive reporting packs</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="34" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>Phase 5</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>17 Sep</t>
-        </is>
-      </c>
-      <c r="C11" s="29" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
-      </c>
-      <c r="D11" s="29" t="inlineStr">
+      <c r="B11" s="31" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C11" s="31" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
         <is>
           <t>Index all outputs; build vector store for semantic search</t>
         </is>
       </c>
-      <c r="E11" s="29" t="inlineStr">
+      <c r="E11" s="32" t="inlineStr">
         <is>
           <t>OpenSearch Serverless, S3</t>
         </is>
       </c>
-      <c r="F11" s="29" t="inlineStr">
+      <c r="F11" s="32" t="inlineStr">
         <is>
           <t>Searchable index</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="34" t="inlineStr">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>Phase 5</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>17 Sep</t>
-        </is>
-      </c>
-      <c r="C12" s="29" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
-      </c>
-      <c r="D12" s="29" t="inlineStr">
+      <c r="B12" s="31" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C12" s="31" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>RAG-based Q&amp;A assistant over organisational memory</t>
         </is>
       </c>
-      <c r="E12" s="29" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr">
         <is>
           <t>Bedrock Knowledge Bases (RAG)</t>
         </is>
       </c>
-      <c r="F12" s="29" t="inlineStr">
+      <c r="F12" s="32" t="inlineStr">
         <is>
           <t>Natural-language Q&amp;A</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="35" t="inlineStr">
+      <c r="A13" s="39" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B13" s="31" t="inlineStr">
-        <is>
-          <t>17 Sep</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
-      </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="B13" s="34" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C13" s="34" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
         <is>
           <t>Design orchestration spine; agent registry &amp; shared data contracts</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr">
+      <c r="E13" s="35" t="inlineStr">
         <is>
           <t>Step Functions, API Gateway</t>
         </is>
       </c>
-      <c r="F13" s="31" t="inlineStr">
+      <c r="F13" s="35" t="inlineStr">
         <is>
           <t>Orchestration design</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="35" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B14" s="31" t="inlineStr">
-        <is>
-          <t>17 Oct</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>16 Nov</t>
-        </is>
-      </c>
-      <c r="D14" s="31" t="inlineStr">
+      <c r="B14" s="34" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C14" s="34" t="n">
+        <v>46342</v>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
         <is>
           <t>Wire all agents together; central console &amp; access control</t>
         </is>
       </c>
-      <c r="E14" s="31" t="inlineStr">
+      <c r="E14" s="35" t="inlineStr">
         <is>
           <t>Bedrock Agents, Cognito</t>
         </is>
       </c>
-      <c r="F14" s="31" t="inlineStr">
+      <c r="F14" s="35" t="inlineStr">
         <is>
           <t>Unified platform</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="35" t="inlineStr">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B15" s="31" t="inlineStr">
-        <is>
-          <t>17 Oct</t>
-        </is>
-      </c>
-      <c r="C15" s="31" t="inlineStr">
-        <is>
-          <t>16 Nov</t>
-        </is>
-      </c>
-      <c r="D15" s="31" t="inlineStr">
+      <c r="B15" s="34" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C15" s="34" t="n">
+        <v>46342</v>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
         <is>
           <t>End-to-end testing, hardening, go-live &amp; handover</t>
         </is>
       </c>
-      <c r="E15" s="31" t="inlineStr">
+      <c r="E15" s="35" t="inlineStr">
         <is>
           <t>CloudWatch, Step Functions</t>
         </is>
       </c>
-      <c r="F15" s="31" t="inlineStr">
+      <c r="F15" s="35" t="inlineStr">
         <is>
           <t>Production Control Tower</t>
         </is>

</xml_diff>